<commit_message>
aligned about this module tab and added scenarios definitions to forecast tab
</commit_message>
<xml_diff>
--- a/data-raw/texts.xlsx
+++ b/data-raw/texts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub_2023\fisheriesXplorer\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E67168F-AD47-4301-8020-C33B61F3F315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E04000-B638-4C78-8867-8090C03733FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30720" yWindow="360" windowWidth="61332" windowHeight="15300" tabRatio="858" firstSheet="21" activeTab="55" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="858" firstSheet="40" activeTab="55" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="overview_AZ" sheetId="8" r:id="rId1"/>
@@ -68,7 +68,8 @@
     <sheet name="bycatch_NrS" sheetId="57" r:id="rId53"/>
     <sheet name="bycatch_NwS" sheetId="58" r:id="rId54"/>
     <sheet name="bycatch_ONA" sheetId="59" r:id="rId55"/>
-    <sheet name="glossary" sheetId="17" r:id="rId56"/>
+    <sheet name="mixfish_scenarios" sheetId="60" r:id="rId56"/>
+    <sheet name="glossary" sheetId="17" r:id="rId57"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -91,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="1013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="1035">
   <si>
     <t>section</t>
   </si>
@@ -4896,6 +4897,72 @@
 Multiannual bycatch rates were estimated for 3 marine mammal species in one métier. The highest bycatch rate was estimated for harbor porpoise in set gillnets, followed by harbor seal in set gillnets and grey seal in set gillnets. &lt;/p&gt;
 &lt;p&gt;
 Multiannual bycatch rates were estimated for 5 seabird species in one métier. The highest bycatch rate was estimated for northern fulmar in set gillnets, followed by common guillemot in set gillnets and razorbill in set gillnets.  &lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Mixed fisheries effort assumption</t>
+  </si>
+  <si>
+    <t>Minimum (min)</t>
+  </si>
+  <si>
+    <t>For each fleet, fishing in forecast year stops when the catch for any one of the stocks meets its stock share. This scenario is the most precautionary option and can highlight some potential “choke species” issues.</t>
+  </si>
+  <si>
+    <t>Maximum (max)</t>
+  </si>
+  <si>
+    <t>For each fleet, fishing in forecast year continues until all its stock shares have been caught. This option illustrates the degree of overshoot of the single-stock advice if fishing is not restricted by the fleet stock shares.</t>
+  </si>
+  <si>
+    <t>Status quo effort (sq_E)</t>
+  </si>
+  <si>
+    <t>The effort of each fleet in forecast year is set equal to the effort in the most recent year (2024).</t>
+  </si>
+  <si>
+    <t>case_study</t>
+  </si>
+  <si>
+    <t>Minimum including ranges (min_range)</t>
+  </si>
+  <si>
+    <t>Same as “min” scenario</t>
+  </si>
+  <si>
+    <t>Minimum excluding zero-catch advice stocks (min_exzero)</t>
+  </si>
+  <si>
+    <t>For each fleet, fishing in forecast year stops when the catch for any one of the stocks meets its stock share, ignoring cod, which has zero- catch advice. This scenario illustrates the effect of fishing on the most limiting stock with non-zero-catch advice.</t>
+  </si>
+  <si>
+    <t>Celtic Sea</t>
+  </si>
+  <si>
+    <t>Greater North Sea</t>
+  </si>
+  <si>
+    <t>Irish Sea</t>
+  </si>
+  <si>
+    <t>Single-stock advice for cod (cod-is), haddock (had-is), Norway lobster (nep-is), sole (sol-is), and whiting (whg-is)</t>
+  </si>
+  <si>
+    <t>For each fleet, fishing in forercast year stops when the catch of the scenario-specified stock meets its stock share. Fleets which do not catch the scenario-specified stock follow a status quo effort assumption (as described for the “sq_E” scenario). In all these single-stock advice scenarios, fleets that target sole (all beam trawls and Belgian otter trawls) are also restricted by their stock share of sole in addition to the scenario-specified stock.</t>
+  </si>
+  <si>
+    <t>Single-stock advice for black-bellied anglerfish (ank-iw), hake (hke-iw), four-spot megrim (ldb-iw), megrim (meg-iw), and white anglerfish (mon-iw)</t>
+  </si>
+  <si>
+    <t>For each fleet, fishing in 2024 stops when the catch of the scenario-specified stock meets its stock share*, regardless of other catches. Fleets which do not catch the scenario-specified stock follow a status quo effort assumption (as described for the “sq_E” scenario).</t>
+  </si>
+  <si>
+    <t>Bay of Biscay</t>
+  </si>
+  <si>
+    <t>Iberian Waters</t>
   </si>
 </sst>
 </file>
@@ -7396,6 +7463,296 @@
 </file>
 
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F161C678-5E6F-46CF-B9B5-1EAF42C93FC4}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="49" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="208.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF5EC4FE-E411-4E36-B8C3-47DB4028DB0F}">
   <dimension ref="A1:C314"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
addedcolumn to scenarios def
</commit_message>
<xml_diff>
--- a/data-raw/texts.xlsx
+++ b/data-raw/texts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub_2023\fisheriesXplorer\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E04000-B638-4C78-8867-8090C03733FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16CB81DB-B56C-456B-8812-7AF1615CAF66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="858" firstSheet="40" activeTab="55" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="1035">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1403" uniqueCount="1040">
   <si>
     <t>section</t>
   </si>
@@ -4963,6 +4963,21 @@
   </si>
   <si>
     <t>Iberian Waters</t>
+  </si>
+  <si>
+    <t>Basis for catch limit in forecast year</t>
+  </si>
+  <si>
+    <t>ICES catch advice</t>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>Catches corresponding to FMSY upper for stocks in good status (SSB ≥ MSY B trigger) and reduced FMSY advice levels (F MSY × SSB/MSY B trigger) for the other stocks (including zero-catch advice).</t>
+  </si>
+  <si>
+    <t>ICES catch advice for stocks with a non- zero-catch advice; no catch limit assumed for stocks with a zero-catch advice.</t>
   </si>
 </sst>
 </file>
@@ -7464,15 +7479,16 @@
 
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F161C678-5E6F-46CF-B9B5-1EAF42C93FC4}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="208.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="91" customWidth="1"/>
+    <col min="3" max="3" width="73.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1013</v>
       </c>
@@ -7480,32 +7496,41 @@
         <v>1014</v>
       </c>
       <c r="C1" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D1" t="s">
         <v>1021</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1015</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1016</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D2" t="s">
         <v>1027</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1017</v>
       </c>
       <c r="B3" t="s">
         <v>1018</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D3" t="s">
         <v>1027</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1019</v>
       </c>
@@ -7513,10 +7538,13 @@
         <v>1020</v>
       </c>
       <c r="C4" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D4" t="s">
         <v>1027</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>1022</v>
       </c>
@@ -7524,10 +7552,13 @@
         <v>1023</v>
       </c>
       <c r="C5" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D5" t="s">
         <v>1027</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>1024</v>
       </c>
@@ -7535,32 +7566,41 @@
         <v>1025</v>
       </c>
       <c r="C6" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D6" t="s">
         <v>1027</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>1015</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>1016</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D7" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>1017</v>
       </c>
       <c r="B8" t="s">
         <v>1018</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D8" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>1019</v>
       </c>
@@ -7568,10 +7608,13 @@
         <v>1020</v>
       </c>
       <c r="C9" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D9" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>1022</v>
       </c>
@@ -7579,43 +7622,52 @@
         <v>1023</v>
       </c>
       <c r="C10" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D10" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>1024</v>
       </c>
       <c r="B11" t="s">
         <v>1025</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>1015</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>1016</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D12" t="s">
         <v>1028</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>1017</v>
       </c>
       <c r="B13" t="s">
         <v>1018</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D13" t="s">
         <v>1028</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>1019</v>
       </c>
@@ -7623,10 +7675,13 @@
         <v>1020</v>
       </c>
       <c r="C14" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D14" t="s">
         <v>1028</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>1022</v>
       </c>
@@ -7634,43 +7689,52 @@
         <v>1023</v>
       </c>
       <c r="C15" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D15" t="s">
         <v>1028</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>1029</v>
       </c>
       <c r="B16" t="s">
         <v>1030</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>1028</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>1015</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>1016</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D17" t="s">
         <v>1034</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>1017</v>
       </c>
       <c r="B18" t="s">
         <v>1018</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D18" t="s">
         <v>1034</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>1019</v>
       </c>
@@ -7678,10 +7742,13 @@
         <v>1020</v>
       </c>
       <c r="C19" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D19" t="s">
         <v>1034</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>1022</v>
       </c>
@@ -7689,43 +7756,55 @@
         <v>1023</v>
       </c>
       <c r="C20" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D20" t="s">
         <v>1034</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>1031</v>
       </c>
       <c r="B21" t="s">
         <v>1032</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D21" t="s">
         <v>1034</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>1015</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>1016</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D22" t="s">
         <v>1033</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>1017</v>
       </c>
       <c r="B23" t="s">
         <v>1018</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D23" t="s">
         <v>1033</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>1019</v>
       </c>
@@ -7733,17 +7812,23 @@
         <v>1020</v>
       </c>
       <c r="C24" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D24" t="s">
         <v>1033</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>1022</v>
       </c>
       <c r="B25" t="s">
         <v>1023</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D25" t="s">
         <v>1033</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ordr of culumn, still a bug to fix but it works
</commit_message>
<xml_diff>
--- a/data-raw/texts.xlsx
+++ b/data-raw/texts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub_2023\fisheriesXplorer\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5843ABC9-0D21-4BD8-91B6-FEF3484894D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A52C6FD-EFB2-47F0-86A2-1786F28C32DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="858" firstSheet="47" activeTab="60" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="858" firstSheet="47" activeTab="55" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="overview_AZ" sheetId="8" r:id="rId1"/>
@@ -7526,7 +7526,7 @@
   <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="49" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="129.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="91" customWidth="1"/>
     <col min="3" max="3" width="73.54296875" customWidth="1"/>
     <col min="4" max="4" width="15.90625" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
updated mixfish text and opened up all sidebars by default
</commit_message>
<xml_diff>
--- a/data-raw/texts.xlsx
+++ b/data-raw/texts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub_2023\fisheriesXplorer\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A52C6FD-EFB2-47F0-86A2-1786F28C32DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D88D8A-559B-42EB-B750-BDF08C3A8C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="858" firstSheet="47" activeTab="55" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="858" firstSheet="48" activeTab="60" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="overview_AZ" sheetId="8" r:id="rId1"/>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1473" uniqueCount="1051">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1473" uniqueCount="1052">
   <si>
     <t>section</t>
   </si>
@@ -5015,7 +5015,10 @@
     <t>Distribution of landings by stock, expressed as a share of total landed weight. Colours identify stocks, and the size of each slice indicates its relative contribution to the landings shown.</t>
   </si>
   <si>
-    <t>lorem ipsum</t>
+    <t>Landings composition in terms of volume by operational mixed-fisheries fleet.</t>
+  </si>
+  <si>
+    <t>Allocation of landings from stocks to operational mixed-fisheries métiers and fleets. The width of each flow is proportional to the landing volume.</t>
   </si>
 </sst>
 </file>
@@ -7942,7 +7945,7 @@
         <v>1045</v>
       </c>
       <c r="B7" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
   </sheetData>
@@ -8013,7 +8016,7 @@
         <v>1045</v>
       </c>
       <c r="B7" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
   </sheetData>
@@ -8082,7 +8085,7 @@
         <v>1045</v>
       </c>
       <c r="B7" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
   </sheetData>
@@ -8206,7 +8209,7 @@
         <v>1045</v>
       </c>
       <c r="B7" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
   </sheetData>
@@ -8275,7 +8278,7 @@
         <v>1045</v>
       </c>
       <c r="B7" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
   </sheetData>

</xml_diff>